<commit_message>
A1: RL B09 results (handoff 24) and the model workbook filled for retail loans: products, salary sources, trend chart
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ability/a1_ability_reference.xlsx
+++ b/docs/ability/a1_ability_reference.xlsx
@@ -640,6 +640,189 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Retail loans: share of accounts by state</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="percentStacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Results trend'!C19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E7D32"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Results trend'!$A$20:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Results trend'!$C$20:$C$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Results trend'!D19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="8BC34A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Results trend'!$A$20:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Results trend'!$D$20:$D$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Results trend'!E19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="D9652B"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Results trend'!$A$20:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Results trend'!$E$20:$E$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Results trend'!F19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="9E9E9E"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Results trend'!$A$20:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Results trend'!$F$20:$F$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <majorUnit val="0.25"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -649,7 +832,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="3060000"/>
+    <ext cx="5400000" cy="2232000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -659,6 +842,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2232000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -957,7 +1162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1048,7 +1253,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10" ht="34" customHeight="1">
       <c r="A10" s="11">
         <f>Results!C6</f>
         <v/>
@@ -1068,310 +1273,346 @@
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12">
-        <f>TEXT(Results!B6,"#,##0")&amp;" cards"&amp;IF(Results!E6="",""," · "&amp;TEXT(Results!E6,"#,##0")&amp;" loans")</f>
+        <f>TEXT(Results!B6,"#,##0")&amp;" credit cards"</f>
         <v/>
       </c>
       <c r="B11" s="12">
-        <f>TEXT(Results!B7,"#,##0")&amp;" cards"&amp;IF(Results!E7="",""," · "&amp;TEXT(Results!E7,"#,##0")&amp;" loans")</f>
+        <f>TEXT(Results!B7,"#,##0")&amp;" credit cards"</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>TEXT(Results!B8,"#,##0")&amp;" cards"&amp;IF(Results!E8="",""," · "&amp;TEXT(Results!E8,"#,##0")&amp;" loans")</f>
+        <f>TEXT(Results!B8,"#,##0")&amp;" credit cards"</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>TEXT(Results!B9,"#,##0")&amp;" cards"&amp;IF(Results!E9="",""," · "&amp;TEXT(Results!E9,"#,##0")&amp;" loans")</f>
+        <f>TEXT(Results!B9,"#,##0")&amp;" credit cards"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="11">
+        <f>Results!E6</f>
+        <v/>
+      </c>
+      <c r="B12" s="11">
+        <f>Results!E7</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>Results!E8</f>
+        <v/>
+      </c>
+      <c r="D12" s="11">
+        <f>Results!E9</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="12">
+        <f>TEXT(Results!D6,"#,##0")&amp;" retail loans"</f>
+        <v/>
+      </c>
+      <c r="B13" s="12">
+        <f>TEXT(Results!D7,"#,##0")&amp;" retail loans"</f>
+        <v/>
+      </c>
+      <c r="C13" s="12">
+        <f>TEXT(Results!D8,"#,##0")&amp;" retail loans"</f>
+        <v/>
+      </c>
+      <c r="D13" s="12">
+        <f>TEXT(Results!D9,"#,##0")&amp;" retail loans"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>States</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Rule</t>
         </is>
       </c>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>In plain words</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="33" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
+    <row r="17" ht="33" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>4 points and no distress</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>Regular income and a buffer, both confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="46.5" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>2–3 points and no distress, or 4 points with distress</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>One side confirmed, or both partly; or everything in place but a payment just failed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="33" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>0–1 points, or under 4 points with distress</t>
         </is>
       </c>
       <c r="C17" s="14" t="n"/>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>What we can see shows little or nothing to pay with.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="33" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>Unknown</t>
+          <t>Regular income and a buffer, both confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46.5" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>0 points, no distress, and no CASA with us or a dormant one</t>
+          <t>2–3 points and no distress, or 4 points with distress</t>
         </is>
       </c>
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="16" t="inlineStr">
         <is>
+          <t>One side confirmed, or both partly; or everything in place but a payment just failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="33" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>0–1 points, or under 4 points with distress</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>What we can see shows little or nothing to pay with.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="33" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>0 points, no distress, and no CASA with us or a dormant one</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
           <t>We cannot see the customer's money.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>State map: income points + liquidity points, then distress</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>No distress</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Liquidity Adequate</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>Liquidity Weak</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Liquidity None</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>Income Stable</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
-        <is>
-          <t>Income Weak</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
+          <t>Income Stable</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>Income Weak</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
           <t>Income None</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>Low (Unknown if CASA dormant or absent)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>With distress</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Liquidity Adequate</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>Liquidity Weak</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Liquidity None</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
-        <is>
-          <t>Income Stable</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>Income Weak</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
+          <t>Income Stable</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>Income Weak</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
           <t>Income None</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C31" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="19.5" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="33" ht="19.5" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Rules: 'Logic'. Which rule gave each state: 'Results detail'. What we can see of the customer: 'Results summaries'.</t>
         </is>
@@ -1381,13 +1622,13 @@
   <mergeCells count="10">
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B14:C14"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="A33:D33"/>
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2981,7 +3222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3078,22 +3319,30 @@
         <f>IF(OR(B6="",N(B$10)=0),"",B6/B$10)</f>
         <v/>
       </c>
-      <c r="D6" s="32" t="n"/>
+      <c r="D6" s="32" t="n">
+        <v>11</v>
+      </c>
       <c r="E6" s="33">
         <f>IF(OR(D6="",N(D$10)=0),"",D6/D$10)</f>
         <v/>
       </c>
-      <c r="F6" s="32" t="n"/>
+      <c r="F6" s="32" t="n">
+        <v>6</v>
+      </c>
       <c r="G6" s="33">
         <f>IF(OR(F6="",N(F$10)=0),"",F6/F$10)</f>
         <v/>
       </c>
-      <c r="H6" s="32" t="n"/>
+      <c r="H6" s="32" t="n">
+        <v>3</v>
+      </c>
       <c r="I6" s="33">
         <f>IF(OR(H6="",N(H$10)=0),"",H6/H$10)</f>
         <v/>
       </c>
-      <c r="J6" s="32" t="n"/>
+      <c r="J6" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="K6" s="33">
         <f>IF(OR(J6="",N(J$10)=0),"",J6/J$10)</f>
         <v/>
@@ -3112,22 +3361,30 @@
         <f>IF(OR(B7="",N(B$10)=0),"",B7/B$10)</f>
         <v/>
       </c>
-      <c r="D7" s="32" t="n"/>
+      <c r="D7" s="32" t="n">
+        <v>358</v>
+      </c>
       <c r="E7" s="33">
         <f>IF(OR(D7="",N(D$10)=0),"",D7/D$10)</f>
         <v/>
       </c>
-      <c r="F7" s="32" t="n"/>
+      <c r="F7" s="32" t="n">
+        <v>100</v>
+      </c>
       <c r="G7" s="33">
         <f>IF(OR(F7="",N(F$10)=0),"",F7/F$10)</f>
         <v/>
       </c>
-      <c r="H7" s="32" t="n"/>
+      <c r="H7" s="32" t="n">
+        <v>134</v>
+      </c>
       <c r="I7" s="33">
         <f>IF(OR(H7="",N(H$10)=0),"",H7/H$10)</f>
         <v/>
       </c>
-      <c r="J7" s="32" t="n"/>
+      <c r="J7" s="32" t="n">
+        <v>124</v>
+      </c>
       <c r="K7" s="33">
         <f>IF(OR(J7="",N(J$10)=0),"",J7/J$10)</f>
         <v/>
@@ -3146,22 +3403,30 @@
         <f>IF(OR(B8="",N(B$10)=0),"",B8/B$10)</f>
         <v/>
       </c>
-      <c r="D8" s="32" t="n"/>
+      <c r="D8" s="32" t="n">
+        <v>1837</v>
+      </c>
       <c r="E8" s="33">
         <f>IF(OR(D8="",N(D$10)=0),"",D8/D$10)</f>
         <v/>
       </c>
-      <c r="F8" s="32" t="n"/>
+      <c r="F8" s="32" t="n">
+        <v>593</v>
+      </c>
       <c r="G8" s="33">
         <f>IF(OR(F8="",N(F$10)=0),"",F8/F$10)</f>
         <v/>
       </c>
-      <c r="H8" s="32" t="n"/>
+      <c r="H8" s="32" t="n">
+        <v>608</v>
+      </c>
       <c r="I8" s="33">
         <f>IF(OR(H8="",N(H$10)=0),"",H8/H$10)</f>
         <v/>
       </c>
-      <c r="J8" s="32" t="n"/>
+      <c r="J8" s="32" t="n">
+        <v>636</v>
+      </c>
       <c r="K8" s="33">
         <f>IF(OR(J8="",N(J$10)=0),"",J8/J$10)</f>
         <v/>
@@ -3180,22 +3445,30 @@
         <f>IF(OR(B9="",N(B$10)=0),"",B9/B$10)</f>
         <v/>
       </c>
-      <c r="D9" s="32" t="n"/>
+      <c r="D9" s="32" t="n">
+        <v>1779</v>
+      </c>
       <c r="E9" s="33">
         <f>IF(OR(D9="",N(D$10)=0),"",D9/D$10)</f>
         <v/>
       </c>
-      <c r="F9" s="32" t="n"/>
+      <c r="F9" s="32" t="n">
+        <v>698</v>
+      </c>
       <c r="G9" s="33">
         <f>IF(OR(F9="",N(F$10)=0),"",F9/F$10)</f>
         <v/>
       </c>
-      <c r="H9" s="32" t="n"/>
+      <c r="H9" s="32" t="n">
+        <v>479</v>
+      </c>
       <c r="I9" s="33">
         <f>IF(OR(H9="",N(H$10)=0),"",H9/H$10)</f>
         <v/>
       </c>
-      <c r="J9" s="32" t="n"/>
+      <c r="J9" s="32" t="n">
+        <v>602</v>
+      </c>
       <c r="K9" s="33">
         <f>IF(OR(J9="",N(J$10)=0),"",J9/J$10)</f>
         <v/>
@@ -3260,7 +3533,7 @@
     <row r="13" ht="33" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>A customer with fewer alerts in the window than before can look like a fall: 912 accounts reach the window total but fail the 25% check. Some are real falls; the data cannot yet split them.</t>
+          <t>A customer with fewer alerts in the window than before can look like a fall: 912 card and 86 loan accounts reach the window total but fail the 25% check. Some are real falls; the data cannot yet split them.</t>
         </is>
       </c>
     </row>
@@ -3288,21 +3561,37 @@
     <row r="17" ht="33" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Internal salary and balances cover the PRB, PSB and PB segments (95% of base customers). Internal salary history starts in September 2024.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+          <t>Every loan customer shows a CASA transaction, so No CASA never fires on loans and all their Unknowns are dormant. The transaction can be just the bank collecting the instalment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="33" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Loan thresholds are higher: one instalment (median AED 2,389) against the card's oldest overdue amount (median AED 837), so a loan salary must cover more to count as Stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="33" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Internal salary and balances cover the PRB, PSB and PB segments (95% of card customers). Internal salary history starts in September 2024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="19.5" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Which rule gave each state: 'Results detail'. Coverage of salary, CASA and bureau: 'Results summaries'.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="15">
     <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A18:K18"/>
     <mergeCell ref="J5:K5"/>
+    <mergeCell ref="A21:K21"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="F5:G5"/>
@@ -3395,7 +3684,9 @@
         <v>19292</v>
       </c>
       <c r="C6" s="36" t="n"/>
-      <c r="D6" s="32" t="n"/>
+      <c r="D6" s="32" t="n">
+        <v>3985</v>
+      </c>
       <c r="E6" s="36" t="n"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
@@ -3411,7 +3702,9 @@
         <f>IF(OR(B7="",N(B$6)=0),"",B7/B$6)</f>
         <v/>
       </c>
-      <c r="D7" s="32" t="n"/>
+      <c r="D7" s="32" t="n">
+        <v>41</v>
+      </c>
       <c r="E7" s="33">
         <f>IF(OR(D7="",N(D$6)=0),"",D7/D$6)</f>
         <v/>
@@ -3430,7 +3723,9 @@
         <f>IF(OR(B8="",N(B$6)=0),"",B8/B$6)</f>
         <v/>
       </c>
-      <c r="D8" s="32" t="n"/>
+      <c r="D8" s="32" t="n">
+        <v>307</v>
+      </c>
       <c r="E8" s="33">
         <f>IF(OR(D8="",N(D$6)=0),"",D8/D$6)</f>
         <v/>
@@ -3449,7 +3744,9 @@
         <f>IF(OR(B9="",N(B$6)=0),"",B9/B$6)</f>
         <v/>
       </c>
-      <c r="D9" s="32" t="n"/>
+      <c r="D9" s="32" t="n">
+        <v>13</v>
+      </c>
       <c r="E9" s="33">
         <f>IF(OR(D9="",N(D$6)=0),"",D9/D$6)</f>
         <v/>
@@ -3468,7 +3765,9 @@
         <f>IF(OR(B10="",N(B$6)=0),"",B10/B$6)</f>
         <v/>
       </c>
-      <c r="D10" s="32" t="n"/>
+      <c r="D10" s="32" t="n">
+        <v>143</v>
+      </c>
       <c r="E10" s="33">
         <f>IF(OR(D10="",N(D$6)=0),"",D10/D$6)</f>
         <v/>
@@ -3487,7 +3786,9 @@
         <f>IF(OR(B11="",N(B$6)=0),"",B11/B$6)</f>
         <v/>
       </c>
-      <c r="D11" s="32" t="n"/>
+      <c r="D11" s="32" t="n">
+        <v>231</v>
+      </c>
       <c r="E11" s="33">
         <f>IF(OR(D11="",N(D$6)=0),"",D11/D$6)</f>
         <v/>
@@ -3506,7 +3807,9 @@
         <f>IF(OR(B12="",N(B$6)=0),"",B12/B$6)</f>
         <v/>
       </c>
-      <c r="D12" s="32" t="n"/>
+      <c r="D12" s="32" t="n">
+        <v>8</v>
+      </c>
       <c r="E12" s="33">
         <f>IF(OR(D12="",N(D$6)=0),"",D12/D$6)</f>
         <v/>
@@ -3525,7 +3828,9 @@
         <f>IF(OR(B13="",N(B$6)=0),"",B13/B$6)</f>
         <v/>
       </c>
-      <c r="D13" s="32" t="n"/>
+      <c r="D13" s="32" t="n">
+        <v>3242</v>
+      </c>
       <c r="E13" s="33">
         <f>IF(OR(D13="",N(D$6)=0),"",D13/D$6)</f>
         <v/>
@@ -3578,7 +3883,9 @@
         <f>IF(OR(B17="",N(B$6)=0),"",B17/B$6)</f>
         <v/>
       </c>
-      <c r="D17" s="32" t="n"/>
+      <c r="D17" s="32" t="n">
+        <v>37</v>
+      </c>
       <c r="E17" s="33">
         <f>IF(OR(D17="",N(D$6)=0),"",D17/D$6)</f>
         <v/>
@@ -3597,7 +3904,9 @@
         <f>IF(OR(B18="",N(B$6)=0),"",B18/B$6)</f>
         <v/>
       </c>
-      <c r="D18" s="32" t="n"/>
+      <c r="D18" s="32" t="n">
+        <v>161</v>
+      </c>
       <c r="E18" s="33">
         <f>IF(OR(D18="",N(D$6)=0),"",D18/D$6)</f>
         <v/>
@@ -3616,7 +3925,9 @@
         <f>IF(OR(B19="",N(B$6)=0),"",B19/B$6)</f>
         <v/>
       </c>
-      <c r="D19" s="32" t="n"/>
+      <c r="D19" s="32" t="n">
+        <v>122</v>
+      </c>
       <c r="E19" s="33">
         <f>IF(OR(D19="",N(D$6)=0),"",D19/D$6)</f>
         <v/>
@@ -3635,7 +3946,9 @@
         <f>IF(OR(B20="",N(B$6)=0),"",B20/B$6)</f>
         <v/>
       </c>
-      <c r="D20" s="32" t="n"/>
+      <c r="D20" s="32" t="n">
+        <v>86</v>
+      </c>
       <c r="E20" s="33">
         <f>IF(OR(D20="",N(D$6)=0),"",D20/D$6)</f>
         <v/>
@@ -3654,7 +3967,9 @@
         <f>IF(OR(B21="",N(B$6)=0),"",B21/B$6)</f>
         <v/>
       </c>
-      <c r="D21" s="32" t="n"/>
+      <c r="D21" s="32" t="n">
+        <v>153</v>
+      </c>
       <c r="E21" s="33">
         <f>IF(OR(D21="",N(D$6)=0),"",D21/D$6)</f>
         <v/>
@@ -3707,7 +4022,9 @@
         <f>IF(OR(B25="",N(B$6)=0),"",B25/B$6)</f>
         <v/>
       </c>
-      <c r="D25" s="32" t="n"/>
+      <c r="D25" s="32" t="n">
+        <v>46</v>
+      </c>
       <c r="E25" s="33">
         <f>IF(OR(D25="",N(D$6)=0),"",D25/D$6)</f>
         <v/>
@@ -3726,7 +4043,9 @@
         <f>IF(OR(B26="",N(B$6)=0),"",B26/B$6)</f>
         <v/>
       </c>
-      <c r="D26" s="32" t="n"/>
+      <c r="D26" s="32" t="n">
+        <v>11</v>
+      </c>
       <c r="E26" s="33">
         <f>IF(OR(D26="",N(D$6)=0),"",D26/D$6)</f>
         <v/>
@@ -3745,7 +4064,9 @@
         <f>IF(OR(B27="",N(B$6)=0),"",B27/B$6)</f>
         <v/>
       </c>
-      <c r="D27" s="32" t="n"/>
+      <c r="D27" s="32" t="n">
+        <v>291</v>
+      </c>
       <c r="E27" s="33">
         <f>IF(OR(D27="",N(D$6)=0),"",D27/D$6)</f>
         <v/>
@@ -3764,7 +4085,9 @@
         <f>IF(OR(B28="",N(B$6)=0),"",B28/B$6)</f>
         <v/>
       </c>
-      <c r="D28" s="32" t="n"/>
+      <c r="D28" s="32" t="n">
+        <v>14</v>
+      </c>
       <c r="E28" s="33">
         <f>IF(OR(D28="",N(D$6)=0),"",D28/D$6)</f>
         <v/>
@@ -3783,7 +4106,9 @@
         <f>IF(OR(B29="",N(B$6)=0),"",B29/B$6)</f>
         <v/>
       </c>
-      <c r="D29" s="32" t="n"/>
+      <c r="D29" s="32" t="n">
+        <v>14</v>
+      </c>
       <c r="E29" s="33">
         <f>IF(OR(D29="",N(D$6)=0),"",D29/D$6)</f>
         <v/>
@@ -3802,7 +4127,9 @@
         <f>IF(OR(B30="",N(B$6)=0),"",B30/B$6)</f>
         <v/>
       </c>
-      <c r="D30" s="32" t="n"/>
+      <c r="D30" s="32" t="n">
+        <v>3609</v>
+      </c>
       <c r="E30" s="33">
         <f>IF(OR(D30="",N(D$6)=0),"",D30/D$6)</f>
         <v/>
@@ -3855,7 +4182,9 @@
         <f>IF(OR(B34="",N(B$6)=0),"",B34/B$6)</f>
         <v/>
       </c>
-      <c r="D34" s="32" t="n"/>
+      <c r="D34" s="32" t="n">
+        <v>3261</v>
+      </c>
       <c r="E34" s="33">
         <f>IF(OR(D34="",N(D$6)=0),"",D34/D$6)</f>
         <v/>
@@ -3874,7 +4203,9 @@
         <f>IF(OR(B35="",N(B$6)=0),"",B35/B$6)</f>
         <v/>
       </c>
-      <c r="D35" s="32" t="n"/>
+      <c r="D35" s="32" t="n">
+        <v>282</v>
+      </c>
       <c r="E35" s="33">
         <f>IF(OR(D35="",N(D$6)=0),"",D35/D$6)</f>
         <v/>
@@ -3893,7 +4224,9 @@
         <f>IF(OR(B36="",N(B$6)=0),"",B36/B$6)</f>
         <v/>
       </c>
-      <c r="D36" s="32" t="n"/>
+      <c r="D36" s="32" t="n">
+        <v>189</v>
+      </c>
       <c r="E36" s="33">
         <f>IF(OR(D36="",N(D$6)=0),"",D36/D$6)</f>
         <v/>
@@ -3912,7 +4245,9 @@
         <f>IF(OR(B37="",N(B$6)=0),"",B37/B$6)</f>
         <v/>
       </c>
-      <c r="D37" s="32" t="n"/>
+      <c r="D37" s="32" t="n">
+        <v>184</v>
+      </c>
       <c r="E37" s="33">
         <f>IF(OR(D37="",N(D$6)=0),"",D37/D$6)</f>
         <v/>
@@ -3931,7 +4266,9 @@
         <f>IF(OR(B38="",N(B$6)=0),"",B38/B$6)</f>
         <v/>
       </c>
-      <c r="D38" s="32" t="n"/>
+      <c r="D38" s="32" t="n">
+        <v>69</v>
+      </c>
       <c r="E38" s="33">
         <f>IF(OR(D38="",N(D$6)=0),"",D38/D$6)</f>
         <v/>
@@ -3984,7 +4321,9 @@
         <f>IF(OR(B42="",N(B$6)=0),"",B42/B$6)</f>
         <v/>
       </c>
-      <c r="D42" s="32" t="n"/>
+      <c r="D42" s="32" t="n">
+        <v>11</v>
+      </c>
       <c r="E42" s="33">
         <f>IF(OR(D42="",N(D$6)=0),"",D42/D$6)</f>
         <v/>
@@ -4003,7 +4342,9 @@
         <f>IF(OR(B43="",N(B$6)=0),"",B43/B$6)</f>
         <v/>
       </c>
-      <c r="D43" s="32" t="n"/>
+      <c r="D43" s="32" t="n">
+        <v>271</v>
+      </c>
       <c r="E43" s="33">
         <f>IF(OR(D43="",N(D$6)=0),"",D43/D$6)</f>
         <v/>
@@ -4022,7 +4363,9 @@
         <f>IF(OR(B44="",N(B$6)=0),"",B44/B$6)</f>
         <v/>
       </c>
-      <c r="D44" s="32" t="n"/>
+      <c r="D44" s="32" t="n">
+        <v>23</v>
+      </c>
       <c r="E44" s="33">
         <f>IF(OR(D44="",N(D$6)=0),"",D44/D$6)</f>
         <v/>
@@ -4041,7 +4384,9 @@
         <f>IF(OR(B45="",N(B$6)=0),"",B45/B$6)</f>
         <v/>
       </c>
-      <c r="D45" s="32" t="n"/>
+      <c r="D45" s="32" t="n">
+        <v>19</v>
+      </c>
       <c r="E45" s="33">
         <f>IF(OR(D45="",N(D$6)=0),"",D45/D$6)</f>
         <v/>
@@ -4060,7 +4405,9 @@
         <f>IF(OR(B46="",N(B$6)=0),"",B46/B$6)</f>
         <v/>
       </c>
-      <c r="D46" s="32" t="n"/>
+      <c r="D46" s="32" t="n">
+        <v>39</v>
+      </c>
       <c r="E46" s="33">
         <f>IF(OR(D46="",N(D$6)=0),"",D46/D$6)</f>
         <v/>
@@ -4079,7 +4426,9 @@
         <f>IF(OR(B47="",N(B$6)=0),"",B47/B$6)</f>
         <v/>
       </c>
-      <c r="D47" s="32" t="n"/>
+      <c r="D47" s="32" t="n">
+        <v>3</v>
+      </c>
       <c r="E47" s="33">
         <f>IF(OR(D47="",N(D$6)=0),"",D47/D$6)</f>
         <v/>
@@ -4098,7 +4447,9 @@
         <f>IF(OR(B48="",N(B$6)=0),"",B48/B$6)</f>
         <v/>
       </c>
-      <c r="D48" s="32" t="n"/>
+      <c r="D48" s="32" t="n">
+        <v>3</v>
+      </c>
       <c r="E48" s="33">
         <f>IF(OR(D48="",N(D$6)=0),"",D48/D$6)</f>
         <v/>
@@ -4151,7 +4502,9 @@
         <f>IF(OR(B52="",N(B$6)=0),"",B52/B$6)</f>
         <v/>
       </c>
-      <c r="D52" s="32" t="n"/>
+      <c r="D52" s="32" t="n">
+        <v>559</v>
+      </c>
       <c r="E52" s="33">
         <f>IF(OR(D52="",N(D$6)=0),"",D52/D$6)</f>
         <v/>
@@ -4170,7 +4523,9 @@
         <f>IF(OR(B53="",N(B$6)=0),"",B53/B$6)</f>
         <v/>
       </c>
-      <c r="D53" s="32" t="n"/>
+      <c r="D53" s="32" t="n">
+        <v>656</v>
+      </c>
       <c r="E53" s="33">
         <f>IF(OR(D53="",N(D$6)=0),"",D53/D$6)</f>
         <v/>
@@ -4189,7 +4544,9 @@
         <f>IF(OR(B54="",N(B$6)=0),"",B54/B$6)</f>
         <v/>
       </c>
-      <c r="D54" s="32" t="n"/>
+      <c r="D54" s="32" t="n">
+        <v>539</v>
+      </c>
       <c r="E54" s="33">
         <f>IF(OR(D54="",N(D$6)=0),"",D54/D$6)</f>
         <v/>
@@ -4208,7 +4565,9 @@
         <f>IF(OR(B55="",N(B$6)=0),"",B55/B$6)</f>
         <v/>
       </c>
-      <c r="D55" s="32" t="n"/>
+      <c r="D55" s="32" t="n">
+        <v>83</v>
+      </c>
       <c r="E55" s="33">
         <f>IF(OR(D55="",N(D$6)=0),"",D55/D$6)</f>
         <v/>
@@ -4261,7 +4620,9 @@
         <f>IF(OR(B59="",N(B$6)=0),"",B59/B$6)</f>
         <v/>
       </c>
-      <c r="D59" s="32" t="n"/>
+      <c r="D59" s="32" t="n">
+        <v>1779</v>
+      </c>
       <c r="E59" s="33">
         <f>IF(OR(D59="",N(D$6)=0),"",D59/D$6)</f>
         <v/>
@@ -4280,16 +4641,18 @@
         <f>IF(OR(B60="",N(B$6)=0),"",B60/B$6)</f>
         <v/>
       </c>
-      <c r="D60" s="32" t="n"/>
+      <c r="D60" s="32" t="n">
+        <v>0</v>
+      </c>
       <c r="E60" s="33">
         <f>IF(OR(D60="",N(D$6)=0),"",D60/D$6)</f>
         <v/>
       </c>
     </row>
-    <row r="62" ht="33" customHeight="1">
+    <row r="62" ht="46.5" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>The AECB Stable and Weak rows include accounts with internal salary too. A card payment can sit beside a sufficient balance, so the arms overlap in the second Adequate row.</t>
+          <t>The AECB Stable and Weak rows include accounts with internal salary too; on loans AECB also includes the salary on the loan's own bureau pull. A card payment can sit beside a sufficient balance, so the arms overlap in the second Adequate row.</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -4504,7 +4867,9 @@
         <v>19292</v>
       </c>
       <c r="C6" s="36" t="n"/>
-      <c r="D6" s="32" t="n"/>
+      <c r="D6" s="32" t="n">
+        <v>3985</v>
+      </c>
       <c r="E6" s="36" t="n"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
@@ -4520,7 +4885,9 @@
         <f>IF(OR(B7="",N(B$6)=0),"",B7/B$6)</f>
         <v/>
       </c>
-      <c r="D7" s="32" t="n"/>
+      <c r="D7" s="32" t="n">
+        <v>1332</v>
+      </c>
       <c r="E7" s="33">
         <f>IF(OR(D7="",N(D$6)=0),"",D7/D$6)</f>
         <v/>
@@ -4539,7 +4906,9 @@
         <f>IF(OR(B8="",N(B$6)=0),"",B8/B$6)</f>
         <v/>
       </c>
-      <c r="D8" s="32" t="n"/>
+      <c r="D8" s="32" t="n">
+        <v>2653</v>
+      </c>
       <c r="E8" s="33">
         <f>IF(OR(D8="",N(D$6)=0),"",D8/D$6)</f>
         <v/>
@@ -4558,7 +4927,9 @@
         <f>IF(OR(B9="",N(B$6)=0),"",B9/B$6)</f>
         <v/>
       </c>
-      <c r="D9" s="32" t="n"/>
+      <c r="D9" s="32" t="n">
+        <v>0</v>
+      </c>
       <c r="E9" s="33">
         <f>IF(OR(D9="",N(D$6)=0),"",D9/D$6)</f>
         <v/>
@@ -4611,7 +4982,9 @@
         <f>IF(OR(B13="",N(B$6)=0),"",B13/B$6)</f>
         <v/>
       </c>
-      <c r="D13" s="32" t="n"/>
+      <c r="D13" s="32" t="n">
+        <v>205</v>
+      </c>
       <c r="E13" s="33">
         <f>IF(OR(D13="",N(D$6)=0),"",D13/D$6)</f>
         <v/>
@@ -4630,7 +5003,9 @@
         <f>IF(OR(B14="",N(B$6)=0),"",B14/B$6)</f>
         <v/>
       </c>
-      <c r="D14" s="32" t="n"/>
+      <c r="D14" s="32" t="n">
+        <v>1146</v>
+      </c>
       <c r="E14" s="33">
         <f>IF(OR(D14="",N(D$6)=0),"",D14/D$6)</f>
         <v/>
@@ -4649,7 +5024,9 @@
         <f>IF(OR(B15="",N(B$6)=0),"",B15/B$6)</f>
         <v/>
       </c>
-      <c r="D15" s="32" t="n"/>
+      <c r="D15" s="32" t="n">
+        <v>888</v>
+      </c>
       <c r="E15" s="33">
         <f>IF(OR(D15="",N(D$6)=0),"",D15/D$6)</f>
         <v/>
@@ -4668,7 +5045,9 @@
         <f>IF(OR(B16="",N(B$6)=0),"",B16/B$6)</f>
         <v/>
       </c>
-      <c r="D16" s="32" t="n"/>
+      <c r="D16" s="32" t="n">
+        <v>528</v>
+      </c>
       <c r="E16" s="33">
         <f>IF(OR(D16="",N(D$6)=0),"",D16/D$6)</f>
         <v/>
@@ -4687,7 +5066,9 @@
         <f>IF(OR(B17="",N(B$6)=0),"",B17/B$6)</f>
         <v/>
       </c>
-      <c r="D17" s="32" t="n"/>
+      <c r="D17" s="32" t="n">
+        <v>1218</v>
+      </c>
       <c r="E17" s="33">
         <f>IF(OR(D17="",N(D$6)=0),"",D17/D$6)</f>
         <v/>
@@ -4740,7 +5121,9 @@
         <f>IF(OR(B21="",N(B$6)=0),"",B21/B$6)</f>
         <v/>
       </c>
-      <c r="D21" s="32" t="n"/>
+      <c r="D21" s="32" t="n">
+        <v>461</v>
+      </c>
       <c r="E21" s="33">
         <f>IF(OR(D21="",N(D$6)=0),"",D21/D$6)</f>
         <v/>
@@ -4759,7 +5142,9 @@
         <f>IF(OR(B22="",N(B$6)=0),"",B22/B$6)</f>
         <v/>
       </c>
-      <c r="D22" s="32" t="n"/>
+      <c r="D22" s="32" t="n">
+        <v>262</v>
+      </c>
       <c r="E22" s="33">
         <f>IF(OR(D22="",N(D$6)=0),"",D22/D$6)</f>
         <v/>
@@ -4778,7 +5163,9 @@
         <f>IF(OR(B23="",N(B$6)=0),"",B23/B$6)</f>
         <v/>
       </c>
-      <c r="D23" s="32" t="n"/>
+      <c r="D23" s="32" t="n">
+        <v>230</v>
+      </c>
       <c r="E23" s="33">
         <f>IF(OR(D23="",N(D$6)=0),"",D23/D$6)</f>
         <v/>
@@ -4797,7 +5184,9 @@
         <f>IF(OR(B24="",N(B$6)=0),"",B24/B$6)</f>
         <v/>
       </c>
-      <c r="D24" s="32" t="n"/>
+      <c r="D24" s="32" t="n">
+        <v>274</v>
+      </c>
       <c r="E24" s="33">
         <f>IF(OR(D24="",N(D$6)=0),"",D24/D$6)</f>
         <v/>
@@ -4816,7 +5205,9 @@
         <f>IF(OR(B25="",N(B$6)=0),"",B25/B$6)</f>
         <v/>
       </c>
-      <c r="D25" s="32" t="n"/>
+      <c r="D25" s="32" t="n">
+        <v>285</v>
+      </c>
       <c r="E25" s="33">
         <f>IF(OR(D25="",N(D$6)=0),"",D25/D$6)</f>
         <v/>
@@ -4835,7 +5226,9 @@
         <f>IF(OR(B26="",N(B$6)=0),"",B26/B$6)</f>
         <v/>
       </c>
-      <c r="D26" s="32" t="n"/>
+      <c r="D26" s="32" t="n">
+        <v>2310</v>
+      </c>
       <c r="E26" s="33">
         <f>IF(OR(D26="",N(D$6)=0),"",D26/D$6)</f>
         <v/>
@@ -4854,7 +5247,9 @@
         <f>IF(OR(B27="",N(B$6)=0),"",B27/B$6)</f>
         <v/>
       </c>
-      <c r="D27" s="32" t="n"/>
+      <c r="D27" s="32" t="n">
+        <v>163</v>
+      </c>
       <c r="E27" s="33">
         <f>IF(OR(D27="",N(D$6)=0),"",D27/D$6)</f>
         <v/>
@@ -4907,7 +5302,9 @@
         <f>IF(OR(B31="",N(B$6)=0),"",B31/B$6)</f>
         <v/>
       </c>
-      <c r="D31" s="32" t="n"/>
+      <c r="D31" s="32" t="n">
+        <v>645</v>
+      </c>
       <c r="E31" s="33">
         <f>IF(OR(D31="",N(D$6)=0),"",D31/D$6)</f>
         <v/>
@@ -4926,7 +5323,9 @@
         <f>IF(OR(B32="",N(B$6)=0),"",B32/B$6)</f>
         <v/>
       </c>
-      <c r="D32" s="32" t="n"/>
+      <c r="D32" s="32" t="n">
+        <v>2615</v>
+      </c>
       <c r="E32" s="33">
         <f>IF(OR(D32="",N(D$6)=0),"",D32/D$6)</f>
         <v/>
@@ -4945,7 +5344,9 @@
         <f>IF(OR(B33="",N(B$6)=0),"",B33/B$6)</f>
         <v/>
       </c>
-      <c r="D33" s="32" t="n"/>
+      <c r="D33" s="32" t="n">
+        <v>725</v>
+      </c>
       <c r="E33" s="33">
         <f>IF(OR(D33="",N(D$6)=0),"",D33/D$6)</f>
         <v/>
@@ -4998,7 +5399,9 @@
         <f>IF(OR(B37="",N(B$6)=0),"",B37/B$6)</f>
         <v/>
       </c>
-      <c r="D37" s="32" t="n"/>
+      <c r="D37" s="32" t="n">
+        <v>1025</v>
+      </c>
       <c r="E37" s="33">
         <f>IF(OR(D37="",N(D$6)=0),"",D37/D$6)</f>
         <v/>
@@ -5017,7 +5420,9 @@
         <f>IF(OR(B38="",N(B$6)=0),"",B38/B$6)</f>
         <v/>
       </c>
-      <c r="D38" s="32" t="n"/>
+      <c r="D38" s="32" t="n">
+        <v>72</v>
+      </c>
       <c r="E38" s="33">
         <f>IF(OR(D38="",N(D$6)=0),"",D38/D$6)</f>
         <v/>
@@ -5036,7 +5441,9 @@
         <f>IF(OR(B39="",N(B$6)=0),"",B39/B$6)</f>
         <v/>
       </c>
-      <c r="D39" s="32" t="n"/>
+      <c r="D39" s="32" t="n">
+        <v>49</v>
+      </c>
       <c r="E39" s="33">
         <f>IF(OR(D39="",N(D$6)=0),"",D39/D$6)</f>
         <v/>
@@ -5055,7 +5462,9 @@
         <f>IF(OR(B40="",N(B$6)=0),"",B40/B$6)</f>
         <v/>
       </c>
-      <c r="D40" s="32" t="n"/>
+      <c r="D40" s="32" t="n">
+        <v>2839</v>
+      </c>
       <c r="E40" s="33">
         <f>IF(OR(D40="",N(D$6)=0),"",D40/D$6)</f>
         <v/>
@@ -5108,7 +5517,9 @@
         <f>IF(OR(B44="",N(B$6)=0),"",B44/B$6)</f>
         <v/>
       </c>
-      <c r="D44" s="32" t="n"/>
+      <c r="D44" s="32" t="n">
+        <v>158</v>
+      </c>
       <c r="E44" s="33">
         <f>IF(OR(D44="",N(D$6)=0),"",D44/D$6)</f>
         <v/>
@@ -5127,7 +5538,9 @@
         <f>IF(OR(B45="",N(B$6)=0),"",B45/B$6)</f>
         <v/>
       </c>
-      <c r="D45" s="32" t="n"/>
+      <c r="D45" s="32" t="n">
+        <v>193</v>
+      </c>
       <c r="E45" s="33">
         <f>IF(OR(D45="",N(D$6)=0),"",D45/D$6)</f>
         <v/>
@@ -5146,7 +5559,9 @@
         <f>IF(OR(B46="",N(B$6)=0),"",B46/B$6)</f>
         <v/>
       </c>
-      <c r="D46" s="32" t="n"/>
+      <c r="D46" s="32" t="n">
+        <v>1410</v>
+      </c>
       <c r="E46" s="33">
         <f>IF(OR(D46="",N(D$6)=0),"",D46/D$6)</f>
         <v/>
@@ -5165,7 +5580,9 @@
         <f>IF(OR(B47="",N(B$6)=0),"",B47/B$6)</f>
         <v/>
       </c>
-      <c r="D47" s="32" t="n"/>
+      <c r="D47" s="32" t="n">
+        <v>2224</v>
+      </c>
       <c r="E47" s="33">
         <f>IF(OR(D47="",N(D$6)=0),"",D47/D$6)</f>
         <v/>
@@ -5218,34 +5635,25 @@
         <f>IF(OR(B51="",N(B$6)=0),"",B51/B$6)</f>
         <v/>
       </c>
-      <c r="D51" s="32" t="n"/>
+      <c r="D51" s="32" t="n">
+        <v>12</v>
+      </c>
       <c r="E51" s="33">
         <f>IF(OR(D51="",N(D$6)=0),"",D51/D$6)</f>
         <v/>
       </c>
     </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Internal salary × AECB salary, credit cards</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>See the sheet 'Salary sources'.</t>
+    <row r="53" ht="19.5" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Internal salary against AECB salary: 'Salary sources'.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A53:E53"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C9">
     <cfRule type="dataBar" priority="1">
@@ -5385,7 +5793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5403,162 +5811,324 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="33" customHeight="1">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Accounts by the latest internal salary and the latest AECB salary alert, credit cards, 31 Aug 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="13" t="inlineStr"/>
-      <c r="B4" s="13" t="inlineStr">
+          <t>Accounts by the latest internal salary and the latest AECB salary alert, 31 Aug 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Credit cards</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="13" t="inlineStr"/>
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>AECB in window</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>AECB 4–6 m</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>AECB 7–12 m</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>AECB 13+ m</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Never</t>
         </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="20" t="inlineStr">
-        <is>
-          <t>Internal in window</t>
-        </is>
-      </c>
-      <c r="B5" s="32" t="n">
-        <v>34</v>
-      </c>
-      <c r="C5" s="32" t="n">
-        <v>15</v>
-      </c>
-      <c r="D5" s="32" t="n">
-        <v>14</v>
-      </c>
-      <c r="E5" s="32" t="n">
-        <v>79</v>
-      </c>
-      <c r="F5" s="32" t="n">
-        <v>298</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>Internal 4–6 m</t>
+          <t>Internal in window</t>
         </is>
       </c>
       <c r="B6" s="32" t="n">
-        <v>349</v>
+        <v>34</v>
       </c>
       <c r="C6" s="32" t="n">
-        <v>121</v>
+        <v>15</v>
       </c>
       <c r="D6" s="32" t="n">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="E6" s="32" t="n">
-        <v>299</v>
+        <v>79</v>
       </c>
       <c r="F6" s="32" t="n">
-        <v>2237</v>
+        <v>298</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
         <is>
-          <t>Internal 7–12 m</t>
+          <t>Internal 4–6 m</t>
         </is>
       </c>
       <c r="B7" s="32" t="n">
-        <v>438</v>
+        <v>349</v>
       </c>
       <c r="C7" s="32" t="n">
-        <v>265</v>
+        <v>121</v>
       </c>
       <c r="D7" s="32" t="n">
-        <v>197</v>
+        <v>88</v>
       </c>
       <c r="E7" s="32" t="n">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="F7" s="32" t="n">
-        <v>2389</v>
+        <v>2237</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>Internal 13–24 m</t>
+          <t>Internal 7–12 m</t>
         </is>
       </c>
       <c r="B8" s="32" t="n">
-        <v>268</v>
+        <v>438</v>
       </c>
       <c r="C8" s="32" t="n">
-        <v>167</v>
+        <v>265</v>
       </c>
       <c r="D8" s="32" t="n">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="E8" s="32" t="n">
-        <v>213</v>
+        <v>310</v>
       </c>
       <c r="F8" s="32" t="n">
-        <v>1104</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
         <is>
+          <t>Internal 13–24 m</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="n">
+        <v>268</v>
+      </c>
+      <c r="C9" s="32" t="n">
+        <v>167</v>
+      </c>
+      <c r="D9" s="32" t="n">
+        <v>189</v>
+      </c>
+      <c r="E9" s="32" t="n">
+        <v>213</v>
+      </c>
+      <c r="F9" s="32" t="n">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
           <t>No internal in 24 m</t>
         </is>
       </c>
-      <c r="B9" s="32" t="n">
+      <c r="B10" s="32" t="n">
         <v>2640</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C10" s="32" t="n">
         <v>1794</v>
       </c>
-      <c r="D9" s="32" t="n">
+      <c r="D10" s="32" t="n">
         <v>1609</v>
       </c>
-      <c r="E9" s="32" t="n">
+      <c r="E10" s="32" t="n">
         <v>1350</v>
       </c>
-      <c r="F9" s="32" t="n">
+      <c r="F10" s="32" t="n">
         <v>2825</v>
       </c>
     </row>
-    <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>'Never' = no AECB salary alert of AED 1,000 or more, with or without alert rows. Retail loans follow.</t>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Retail loans</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="13" t="inlineStr"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>AECB in window</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>AECB 4–6 m</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>AECB 7–12 m</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>AECB 13+ m</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>Internal in window</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="n">
+        <v>21</v>
+      </c>
+      <c r="C14" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="32" t="n">
+        <v>29</v>
+      </c>
+      <c r="F14" s="32" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Internal 4–6 m</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="n">
+        <v>93</v>
+      </c>
+      <c r="C15" s="32" t="n">
+        <v>47</v>
+      </c>
+      <c r="D15" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="E15" s="32" t="n">
+        <v>178</v>
+      </c>
+      <c r="F15" s="32" t="n">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Internal 7–12 m</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="n">
+        <v>108</v>
+      </c>
+      <c r="C16" s="32" t="n">
+        <v>62</v>
+      </c>
+      <c r="D16" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="E16" s="32" t="n">
+        <v>136</v>
+      </c>
+      <c r="F16" s="32" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>Internal 13–24 m</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="n">
+        <v>91</v>
+      </c>
+      <c r="C17" s="32" t="n">
+        <v>49</v>
+      </c>
+      <c r="D17" s="32" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" s="32" t="n">
+        <v>76</v>
+      </c>
+      <c r="F17" s="32" t="n">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>No internal in 24 m</t>
+        </is>
+      </c>
+      <c r="B18" s="32" t="n">
+        <v>148</v>
+      </c>
+      <c r="C18" s="32" t="n">
+        <v>103</v>
+      </c>
+      <c r="D18" s="32" t="n">
+        <v>102</v>
+      </c>
+      <c r="E18" s="32" t="n">
+        <v>140</v>
+      </c>
+      <c r="F18" s="32" t="n">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="20" ht="33" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>'Never' = no AECB salary alert of AED 1,000 or more, with or without alert rows. Before the 1-month carry.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A20:F20"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5572,7 +6142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5817,157 +6387,237 @@
         <v>0.5608</v>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Retail loans 61–180</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Accounts</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="34" t="inlineStr">
-        <is>
-          <t>Jan 2026</t>
-        </is>
-      </c>
-      <c r="B17" s="32" t="n"/>
-      <c r="C17" s="37" t="n"/>
-      <c r="D17" s="37" t="n"/>
-      <c r="E17" s="37" t="n"/>
-      <c r="F17" s="37" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="34" t="inlineStr">
-        <is>
-          <t>Feb 2026</t>
-        </is>
-      </c>
-      <c r="B18" s="32" t="n"/>
-      <c r="C18" s="37" t="n"/>
-      <c r="D18" s="37" t="n"/>
-      <c r="E18" s="37" t="n"/>
-      <c r="F18" s="37" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="34" t="inlineStr">
-        <is>
-          <t>Mar 2026</t>
-        </is>
-      </c>
-      <c r="B19" s="32" t="n"/>
-      <c r="C19" s="37" t="n"/>
-      <c r="D19" s="37" t="n"/>
-      <c r="E19" s="37" t="n"/>
-      <c r="F19" s="37" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="34" t="inlineStr">
         <is>
-          <t>Apr 2026</t>
-        </is>
-      </c>
-      <c r="B20" s="32" t="n"/>
-      <c r="C20" s="37" t="n"/>
-      <c r="D20" s="37" t="n"/>
-      <c r="E20" s="37" t="n"/>
-      <c r="F20" s="37" t="n"/>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="B20" s="32" t="n">
+        <v>2324</v>
+      </c>
+      <c r="C20" s="37" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="D20" s="37" t="n">
+        <v>0.1256</v>
+      </c>
+      <c r="E20" s="37" t="n">
+        <v>0.4617</v>
+      </c>
+      <c r="F20" s="37" t="n">
+        <v>0.4122</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="34" t="inlineStr">
         <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="B21" s="32" t="n"/>
-      <c r="C21" s="37" t="n"/>
-      <c r="D21" s="37" t="n"/>
-      <c r="E21" s="37" t="n"/>
-      <c r="F21" s="37" t="n"/>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="n">
+        <v>2213</v>
+      </c>
+      <c r="C21" s="37" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="D21" s="37" t="n">
+        <v>0.1094</v>
+      </c>
+      <c r="E21" s="37" t="n">
+        <v>0.4424</v>
+      </c>
+      <c r="F21" s="37" t="n">
+        <v>0.4474</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="34" t="inlineStr">
         <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="B22" s="32" t="n"/>
-      <c r="C22" s="37" t="n"/>
-      <c r="D22" s="37" t="n"/>
-      <c r="E22" s="37" t="n"/>
-      <c r="F22" s="37" t="n"/>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B22" s="32" t="n">
+        <v>2218</v>
+      </c>
+      <c r="C22" s="37" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="D22" s="37" t="n">
+        <v>0.1123</v>
+      </c>
+      <c r="E22" s="37" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="F22" s="37" t="n">
+        <v>0.4274</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="34" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
-        </is>
-      </c>
-      <c r="B23" s="32" t="n"/>
-      <c r="C23" s="37" t="n"/>
-      <c r="D23" s="37" t="n"/>
-      <c r="E23" s="37" t="n"/>
-      <c r="F23" s="37" t="n"/>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B23" s="32" t="n">
+        <v>2661</v>
+      </c>
+      <c r="C23" s="37" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="D23" s="37" t="n">
+        <v>0.1184</v>
+      </c>
+      <c r="E23" s="37" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="F23" s="37" t="n">
+        <v>0.4021</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="34" t="inlineStr">
         <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B24" s="32" t="n">
+        <v>3096</v>
+      </c>
+      <c r="C24" s="37" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D24" s="37" t="n">
+        <v>0.1153</v>
+      </c>
+      <c r="E24" s="37" t="n">
+        <v>0.491</v>
+      </c>
+      <c r="F24" s="37" t="n">
+        <v>0.3928</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="34" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="n">
+        <v>3514</v>
+      </c>
+      <c r="C25" s="37" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="D25" s="37" t="n">
+        <v>0.1033</v>
+      </c>
+      <c r="E25" s="37" t="n">
+        <v>0.488</v>
+      </c>
+      <c r="F25" s="37" t="n">
+        <v>0.4069</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="n">
+        <v>3728</v>
+      </c>
+      <c r="C26" s="37" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="D26" s="37" t="n">
+        <v>0.09630000000000001</v>
+      </c>
+      <c r="E26" s="37" t="n">
+        <v>0.4742</v>
+      </c>
+      <c r="F26" s="37" t="n">
+        <v>0.4286</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="34" t="inlineStr">
+        <is>
           <t>Aug 2026</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n"/>
-      <c r="C24" s="37" t="n"/>
-      <c r="D24" s="37" t="n"/>
-      <c r="E24" s="37" t="n"/>
-      <c r="F24" s="37" t="n"/>
-    </row>
-    <row r="26" ht="33" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>The book grows from May. Moderate falls steadily, and August also has slightly short alert data ('Results').</t>
+      <c r="B27" s="32" t="n">
+        <v>3985</v>
+      </c>
+      <c r="C27" s="37" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="D27" s="37" t="n">
+        <v>0.0898</v>
+      </c>
+      <c r="E27" s="37" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="F27" s="37" t="n">
+        <v>0.4464</v>
+      </c>
+    </row>
+    <row r="29" ht="46.5" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Both books grow from April–May while Moderate falls and Unknown rises from June. August also has slightly short alert data ('Results'). High is too small to read on the charts.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A29:F29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>